<commit_message>
Added midterm 1 solution
</commit_message>
<xml_diff>
--- a/Homework 1/HW1 part 2 solution.xlsx
+++ b/Homework 1/HW1 part 2 solution.xlsx
@@ -34720,19 +34720,19 @@
         <v>14</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C10" s="1" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>3</v>
       </c>
       <c r="E10" s="1" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>